<commit_message>
Added regex messages to all constants files and updated create-post.dto.ts.
</commit_message>
<xml_diff>
--- a/Portal_Database_Design/happy_&_sad_paths/List_Of_Regexes.xlsx
+++ b/Portal_Database_Design/happy_&_sad_paths/List_Of_Regexes.xlsx
@@ -199,7 +199,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -234,16 +234,6 @@
       <family val="1"/>
       <charset val="1"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -287,7 +277,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -304,19 +294,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -506,7 +488,7 @@
       <c r="B4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D4" s="1" t="s">
@@ -529,7 +511,7 @@
       <c r="D5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="5" t="s">
         <v>17</v>
       </c>
     </row>
@@ -540,13 +522,13 @@
       <c r="B6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="5" t="s">
         <v>17</v>
       </c>
     </row>
@@ -557,13 +539,13 @@
       <c r="B7" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="5" t="s">
         <v>22</v>
       </c>
     </row>
@@ -580,7 +562,7 @@
       <c r="D8" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="5" t="s">
         <v>27</v>
       </c>
     </row>
@@ -597,7 +579,7 @@
       <c r="D9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="5" t="s">
         <v>31</v>
       </c>
     </row>
@@ -648,7 +630,7 @@
       <c r="D12" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="5" t="s">
         <v>40</v>
       </c>
     </row>
@@ -665,7 +647,7 @@
       <c r="D13" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="5" t="s">
         <v>45</v>
       </c>
     </row>

</xml_diff>